<commit_message>
[SCRUM MASTER] Updated the Burndown Chart, Gantt Chart and Scrum Board to reflect the current state of the sprint.
</commit_message>
<xml_diff>
--- a/SE202526/Management/Burndown Chart.xlsx
+++ b/SE202526/Management/Burndown Chart.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilh\Documents\Universidade\ES\Projeto\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B8CEC3-265B-4E97-BA6C-5F2E2DD5BC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3900FA-4D84-4E49-8762-D8051B0A6729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Burndown Chart" sheetId="1" r:id="rId1"/>
+    <sheet name="Burndown Chart Sprint 5" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="24">
   <si>
     <t>Sprint Burndown Chart</t>
   </si>
@@ -77,6 +78,21 @@
     <t>Dia 8</t>
   </si>
   <si>
+    <t>Find Code Smells</t>
+  </si>
+  <si>
+    <t>Find Design Patterns</t>
+  </si>
+  <si>
+    <t>Create Use Cases</t>
+  </si>
+  <si>
+    <t>Produce Code Metrics</t>
+  </si>
+  <si>
+    <t>Review Work</t>
+  </si>
+  <si>
     <t>Esforço Completo</t>
   </si>
   <si>
@@ -108,22 +124,21 @@
     </r>
   </si>
   <si>
-    <t>Plan upgrades for user stories</t>
+    <t>Analyze the code relative to the two first User Stories</t>
   </si>
   <si>
-    <t>Review code and documenting</t>
+    <t>Implement User Stories 1 and 2</t>
   </si>
   <si>
-    <t>Implementing</t>
+    <t>Produce videos/tests and documentation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mmm/yy"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -677,6 +692,27 @@
   </cellStyleXfs>
   <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -689,13 +725,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -788,50 +824,29 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1077,25 +1092,25 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.5</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>1</c:v>
@@ -1105,7 +1120,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-644A-42BA-A876-FB0052D82B52}"/>
+              <c16:uniqueId val="{00000000-52DF-4757-8C4E-97B55E1A481E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1239,31 +1254,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0" formatCode="General">
-                  <c:v>20</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>20</c:v>
+                  <c:v>7.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14.5</c:v>
+                  <c:v>7.1999999999999993</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11.5</c:v>
+                  <c:v>6.3999999999999995</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>10.5</c:v>
+                  <c:v>5.8</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8.5</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.5</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1271,7 +1286,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-644A-42BA-A876-FB0052D82B52}"/>
+              <c16:uniqueId val="{00000001-52DF-4757-8C4E-97B55E1A481E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1383,31 +1398,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0" formatCode="General">
-                  <c:v>20</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>7.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>6.4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14</c:v>
+                  <c:v>5.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12</c:v>
+                  <c:v>4.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>10</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8</c:v>
+                  <c:v>3.1999999999999993</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>2.3999999999999995</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4</c:v>
+                  <c:v>1.5999999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1415,7 +1430,722 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-644A-42BA-A876-FB0052D82B52}"/>
+              <c16:uniqueId val="{00000002-52DF-4757-8C4E-97B55E1A481E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="36659859"/>
+        <c:axId val="10455904"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="36659859"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8B8B8B"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="10455904"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="10455904"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="22"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6480">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="pt-PT" sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Calibri"/>
+                    <a:ea typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Horas</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8B8B8B"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="36659859"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+              <a:ea typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-PT" sz="1400" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Sprint Burndown Chart</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Esforço Completo</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFC000"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Calibri"/>
+                    <a:ea typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="0">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                    </a:ln>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Burndown Chart Sprint 5'!$D$5:$L$5</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Dia 0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Dia 1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dia 2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dia 3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Dia 4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Dia 5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Dia 6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Dia 7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Dia 8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Burndown Chart Sprint 5'!$D$20:$L$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4E5C-497D-B1A4-B35278365936}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="36659859"/>
+        <c:axId val="10455904"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Esforço Restante</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Calibri"/>
+                    <a:ea typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="28440">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                    </a:ln>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Burndown Chart Sprint 5'!$D$5:$L$5</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Dia 0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Dia 1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dia 2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dia 3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Dia 4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Dia 5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Dia 6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Dia 7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Dia 8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Burndown Chart Sprint 5'!$D$21:$L$21</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-4E5C-497D-B1A4-B35278365936}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Burndown Ideal</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Calibri"/>
+                    <a:ea typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="28440">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                    </a:ln>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Burndown Chart Sprint 5'!$D$5:$L$5</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Dia 0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Dia 1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dia 2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dia 3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Dia 4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Dia 5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Dia 6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Dia 7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Dia 8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Burndown Chart Sprint 5'!$D$22:$L$22</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17.100000000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11.4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.6000000000000014</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.7000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.8000000000000007</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-4E5C-497D-B1A4-B35278365936}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1667,6 +2397,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9360</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>367200</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>171000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F642068-F88C-4308-A53B-7B63A3BEEAA7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -1856,492 +2629,476 @@
   <sheetData>
     <row r="1" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
     </row>
     <row r="3" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="5"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="12"/>
     </row>
     <row r="4" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="53" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7">
-        <v>45971</v>
-      </c>
-      <c r="F4" s="7">
-        <v>45972</v>
-      </c>
-      <c r="G4" s="7">
-        <v>45973</v>
-      </c>
-      <c r="H4" s="7">
-        <v>45974</v>
-      </c>
-      <c r="I4" s="7">
-        <v>45975</v>
-      </c>
-      <c r="J4" s="8">
-        <v>45976</v>
-      </c>
-      <c r="K4" s="7">
-        <v>45977</v>
-      </c>
-      <c r="L4" s="9">
-        <v>45978</v>
+      <c r="E4" s="14">
+        <v>45961</v>
+      </c>
+      <c r="F4" s="14">
+        <v>45962</v>
+      </c>
+      <c r="G4" s="14">
+        <v>45963</v>
+      </c>
+      <c r="H4" s="14">
+        <v>45964</v>
+      </c>
+      <c r="I4" s="14">
+        <v>45965</v>
+      </c>
+      <c r="J4" s="15">
+        <v>45966</v>
+      </c>
+      <c r="K4" s="14">
+        <v>45967</v>
+      </c>
+      <c r="L4" s="16">
+        <v>45968</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="52"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="10" t="s">
+      <c r="B5" s="5"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="12" t="s">
+      <c r="J5" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K5" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="L5" s="20" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="14">
+      <c r="B6" s="21">
         <v>1</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="16">
-        <v>6</v>
-      </c>
-      <c r="E6" s="17">
-        <v>0</v>
-      </c>
-      <c r="F6" s="17">
-        <v>2</v>
-      </c>
-      <c r="G6" s="17">
-        <v>3</v>
-      </c>
-      <c r="H6" s="17">
+      <c r="C6" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="23">
         <v>1</v>
       </c>
-      <c r="I6" s="17">
-        <v>0</v>
-      </c>
-      <c r="J6" s="18">
-        <v>0</v>
-      </c>
-      <c r="K6" s="17">
-        <v>0</v>
-      </c>
-      <c r="L6" s="19">
-        <v>0</v>
-      </c>
+      <c r="E6" s="24">
+        <v>0.2</v>
+      </c>
+      <c r="F6" s="24">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="24">
+        <v>0.2</v>
+      </c>
+      <c r="H6" s="24">
+        <v>0.4</v>
+      </c>
+      <c r="I6" s="24"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="26"/>
     </row>
     <row r="7" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="20">
+      <c r="B7" s="27">
         <v>2</v>
       </c>
-      <c r="C7" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="22">
-        <v>10</v>
-      </c>
-      <c r="E7" s="23">
-        <v>0</v>
-      </c>
-      <c r="F7" s="23">
-        <v>0</v>
-      </c>
-      <c r="G7" s="23">
-        <v>0.5</v>
-      </c>
-      <c r="H7" s="23">
-        <v>2</v>
-      </c>
-      <c r="I7" s="23">
+      <c r="C7" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="29">
+        <v>3</v>
+      </c>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30">
+        <v>0.2</v>
+      </c>
+      <c r="H7" s="30">
+        <v>0.4</v>
+      </c>
+      <c r="I7" s="30">
+        <v>0.6</v>
+      </c>
+      <c r="J7" s="31">
+        <v>0.8</v>
+      </c>
+      <c r="K7" s="30">
         <v>1</v>
       </c>
-      <c r="J7" s="24">
-        <v>2</v>
-      </c>
-      <c r="K7" s="23">
-        <v>1</v>
-      </c>
-      <c r="L7" s="25">
-        <v>1</v>
-      </c>
+      <c r="L7" s="32"/>
     </row>
     <row r="8" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20">
+      <c r="B8" s="27">
         <v>3</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="22">
-        <v>4</v>
-      </c>
-      <c r="E8" s="23">
-        <v>0</v>
-      </c>
-      <c r="F8" s="23">
-        <v>0</v>
-      </c>
-      <c r="G8" s="23">
-        <v>0</v>
-      </c>
-      <c r="H8" s="23">
-        <v>0</v>
-      </c>
-      <c r="I8" s="23">
-        <v>0</v>
-      </c>
-      <c r="J8" s="24">
-        <v>0</v>
-      </c>
-      <c r="K8" s="23">
-        <v>0</v>
-      </c>
-      <c r="L8" s="25">
-        <v>0</v>
-      </c>
+      <c r="C8" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="29">
+        <v>1</v>
+      </c>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="31">
+        <v>1</v>
+      </c>
+      <c r="K8" s="30"/>
+      <c r="L8" s="32"/>
     </row>
     <row r="9" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="20">
+      <c r="B9" s="27">
         <v>4</v>
       </c>
-      <c r="C9" s="26"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="25"/>
+      <c r="C9" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="29">
+        <v>2</v>
+      </c>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="30">
+        <v>2</v>
+      </c>
+      <c r="L9" s="32"/>
     </row>
     <row r="10" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="20">
+      <c r="B10" s="27">
         <v>5</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="25"/>
+      <c r="C10" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="29">
+        <v>1</v>
+      </c>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="32">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="20">
+      <c r="B11" s="27">
         <v>6</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="25"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="32"/>
     </row>
     <row r="12" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="20">
+      <c r="B12" s="27">
         <v>7</v>
       </c>
-      <c r="C12" s="27"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="25"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="32"/>
     </row>
     <row r="13" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="20">
+      <c r="B13" s="27">
         <v>8</v>
       </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="25"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="32"/>
     </row>
     <row r="14" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="20">
+      <c r="B14" s="27">
         <v>9</v>
       </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="25"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="32"/>
     </row>
     <row r="15" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="20">
+      <c r="B15" s="27">
         <v>10</v>
       </c>
-      <c r="C15" s="27"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="25"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="32"/>
     </row>
     <row r="16" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="20">
+      <c r="B16" s="27">
         <v>11</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="25"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="32"/>
     </row>
     <row r="17" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="20">
+      <c r="B17" s="27">
         <v>12</v>
       </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="24"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="25"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="32"/>
     </row>
     <row r="18" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="20">
+      <c r="B18" s="27">
         <v>13</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="25"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="32"/>
     </row>
     <row r="19" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="29">
+      <c r="B19" s="36">
         <v>14</v>
       </c>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="34"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="39"/>
+      <c r="I19" s="39"/>
+      <c r="J19" s="40"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="41"/>
     </row>
     <row r="20" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="54" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="35">
+      <c r="B20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="42">
         <v>0</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="43">
         <f t="shared" ref="E20:L20" si="0">SUM(E6:E19)</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="F20" s="43">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="G20" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="G20" s="43">
         <f t="shared" si="0"/>
-        <v>3.5</v>
-      </c>
-      <c r="H20" s="36">
+        <v>0.4</v>
+      </c>
+      <c r="H20" s="43">
+        <f t="shared" si="0"/>
+        <v>0.8</v>
+      </c>
+      <c r="I20" s="43">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+      <c r="J20" s="44">
+        <f t="shared" si="0"/>
+        <v>1.8</v>
+      </c>
+      <c r="K20" s="44">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="I20" s="36">
+      <c r="L20" s="45">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="J20" s="37">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="K20" s="37">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L20" s="38">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
     </row>
     <row r="21" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="48" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="39">
+      <c r="B21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="46">
         <f>SUM(D6:D20)</f>
-        <v>20</v>
-      </c>
-      <c r="E21" s="40">
+        <v>8</v>
+      </c>
+      <c r="E21" s="47">
         <f t="shared" ref="E21:L21" si="1">D21-SUM(E6:E19)</f>
-        <v>20</v>
-      </c>
-      <c r="F21" s="40">
+        <v>7.8</v>
+      </c>
+      <c r="F21" s="47">
         <f t="shared" si="1"/>
-        <v>18</v>
-      </c>
-      <c r="G21" s="40">
+        <v>7.6</v>
+      </c>
+      <c r="G21" s="47">
         <f t="shared" si="1"/>
-        <v>14.5</v>
-      </c>
-      <c r="H21" s="40">
+        <v>7.1999999999999993</v>
+      </c>
+      <c r="H21" s="47">
         <f t="shared" si="1"/>
-        <v>11.5</v>
-      </c>
-      <c r="I21" s="40">
+        <v>6.3999999999999995</v>
+      </c>
+      <c r="I21" s="47">
         <f t="shared" si="1"/>
-        <v>10.5</v>
-      </c>
-      <c r="J21" s="41">
+        <v>5.8</v>
+      </c>
+      <c r="J21" s="48">
         <f t="shared" si="1"/>
-        <v>8.5</v>
-      </c>
-      <c r="K21" s="42">
+        <v>4</v>
+      </c>
+      <c r="K21" s="49">
         <f t="shared" si="1"/>
-        <v>7.5</v>
-      </c>
-      <c r="L21" s="43">
+        <v>1</v>
+      </c>
+      <c r="L21" s="50">
         <f t="shared" si="1"/>
-        <v>6.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="49" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="49"/>
-      <c r="D22" s="44">
+      <c r="B22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="1"/>
+      <c r="D22" s="51">
         <f>D21</f>
-        <v>20</v>
-      </c>
-      <c r="E22" s="45">
+        <v>8</v>
+      </c>
+      <c r="E22" s="52">
         <f>$D$22-($D$22/10*1)</f>
-        <v>18</v>
-      </c>
-      <c r="F22" s="45">
+        <v>7.2</v>
+      </c>
+      <c r="F22" s="52">
         <f>$D$22-($D$22/10*2)</f>
-        <v>16</v>
-      </c>
-      <c r="G22" s="45">
+        <v>6.4</v>
+      </c>
+      <c r="G22" s="52">
         <f>$D$22-($D$22/10*3)</f>
-        <v>14</v>
-      </c>
-      <c r="H22" s="45">
+        <v>5.6</v>
+      </c>
+      <c r="H22" s="52">
         <f>$D$22-($D$22/10*4)</f>
-        <v>12</v>
-      </c>
-      <c r="I22" s="45">
+        <v>4.8</v>
+      </c>
+      <c r="I22" s="52">
         <f>$D$22-($D$22/10*5)</f>
-        <v>10</v>
-      </c>
-      <c r="J22" s="46">
+        <v>4</v>
+      </c>
+      <c r="J22" s="53">
         <f>$D$22-($D$22/10*6)</f>
-        <v>8</v>
-      </c>
-      <c r="K22" s="45">
+        <v>3.1999999999999993</v>
+      </c>
+      <c r="K22" s="52">
         <f>$D$22-($D$22/10*7)</f>
-        <v>6</v>
-      </c>
-      <c r="L22" s="47">
+        <v>2.3999999999999995</v>
+      </c>
+      <c r="L22" s="54">
         <f>$D$22-($D$22/10*8)</f>
-        <v>4</v>
+        <v>1.5999999999999996</v>
       </c>
     </row>
     <row r="23" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -3336,4 +4093,1468 @@
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDEF1E91-1F52-494C-B1A2-6E397623B912}">
+  <dimension ref="B1:L1000"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" customWidth="1"/>
+    <col min="2" max="2" width="7.1796875" customWidth="1"/>
+    <col min="3" max="3" width="73.08984375" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" customWidth="1"/>
+    <col min="5" max="14" width="10" customWidth="1"/>
+    <col min="15" max="26" width="8.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+    </row>
+    <row r="3" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="8"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="12"/>
+    </row>
+    <row r="4" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="14">
+        <v>45979</v>
+      </c>
+      <c r="F4" s="14">
+        <v>45980</v>
+      </c>
+      <c r="G4" s="14">
+        <v>45981</v>
+      </c>
+      <c r="H4" s="14">
+        <v>45982</v>
+      </c>
+      <c r="I4" s="14">
+        <v>45983</v>
+      </c>
+      <c r="J4" s="14">
+        <v>45984</v>
+      </c>
+      <c r="K4" s="14">
+        <v>45985</v>
+      </c>
+      <c r="L4" s="14">
+        <v>45986</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="5"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="21">
+        <v>1</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="23">
+        <v>6</v>
+      </c>
+      <c r="E6" s="24">
+        <v>1</v>
+      </c>
+      <c r="F6" s="24">
+        <v>3</v>
+      </c>
+      <c r="G6" s="24">
+        <v>2</v>
+      </c>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="26"/>
+    </row>
+    <row r="7" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="27">
+        <v>2</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="29">
+        <v>7</v>
+      </c>
+      <c r="E7" s="30">
+        <v>2</v>
+      </c>
+      <c r="F7" s="30">
+        <v>3</v>
+      </c>
+      <c r="G7" s="30">
+        <v>5</v>
+      </c>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="32"/>
+    </row>
+    <row r="8" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="27">
+        <v>3</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="29">
+        <v>4</v>
+      </c>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="32"/>
+    </row>
+    <row r="9" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="27">
+        <v>4</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="29">
+        <v>2</v>
+      </c>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="32"/>
+    </row>
+    <row r="10" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="27">
+        <v>5</v>
+      </c>
+      <c r="D10" s="29"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="32"/>
+    </row>
+    <row r="11" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="27">
+        <v>6</v>
+      </c>
+      <c r="C11" s="34"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="32"/>
+    </row>
+    <row r="12" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="27">
+        <v>7</v>
+      </c>
+      <c r="C12" s="34"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="32"/>
+    </row>
+    <row r="13" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="27">
+        <v>8</v>
+      </c>
+      <c r="C13" s="34"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="32"/>
+    </row>
+    <row r="14" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="27">
+        <v>9</v>
+      </c>
+      <c r="C14" s="34"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="32"/>
+    </row>
+    <row r="15" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="27">
+        <v>10</v>
+      </c>
+      <c r="C15" s="34"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="32"/>
+    </row>
+    <row r="16" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="27">
+        <v>11</v>
+      </c>
+      <c r="C16" s="35"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="32"/>
+    </row>
+    <row r="17" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="27">
+        <v>12</v>
+      </c>
+      <c r="C17" s="34"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="32"/>
+    </row>
+    <row r="18" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="27">
+        <v>13</v>
+      </c>
+      <c r="C18" s="34"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="32"/>
+    </row>
+    <row r="19" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B19" s="36">
+        <v>14</v>
+      </c>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="39"/>
+      <c r="I19" s="39"/>
+      <c r="J19" s="40"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="41"/>
+    </row>
+    <row r="20" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="42">
+        <v>0</v>
+      </c>
+      <c r="E20" s="43">
+        <f t="shared" ref="E20:L20" si="0">SUM(E6:E19)</f>
+        <v>3</v>
+      </c>
+      <c r="F20" s="43">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="G20" s="43">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="H20" s="43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="44">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K20" s="44">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L20" s="45">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="46">
+        <f>SUM(D6:D20)</f>
+        <v>19</v>
+      </c>
+      <c r="E21" s="47">
+        <f t="shared" ref="E21:L21" si="1">D21-SUM(E6:E19)</f>
+        <v>16</v>
+      </c>
+      <c r="F21" s="47">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="G21" s="47">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="H21" s="47">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="I21" s="47">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="J21" s="48">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="K21" s="49">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="L21" s="50">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="1"/>
+      <c r="D22" s="51">
+        <f>D21</f>
+        <v>19</v>
+      </c>
+      <c r="E22" s="52">
+        <f>$D$22-($D$22/10*1)</f>
+        <v>17.100000000000001</v>
+      </c>
+      <c r="F22" s="52">
+        <f>$D$22-($D$22/10*2)</f>
+        <v>15.2</v>
+      </c>
+      <c r="G22" s="52">
+        <f>$D$22-($D$22/10*3)</f>
+        <v>13.3</v>
+      </c>
+      <c r="H22" s="52">
+        <f>$D$22-($D$22/10*4)</f>
+        <v>11.4</v>
+      </c>
+      <c r="I22" s="52">
+        <f>$D$22-($D$22/10*5)</f>
+        <v>9.5</v>
+      </c>
+      <c r="J22" s="53">
+        <f>$D$22-($D$22/10*6)</f>
+        <v>7.6000000000000014</v>
+      </c>
+      <c r="K22" s="52">
+        <f>$D$22-($D$22/10*7)</f>
+        <v>5.7000000000000011</v>
+      </c>
+      <c r="L22" s="54">
+        <f>$D$22-($D$22/10*8)</f>
+        <v>3.8000000000000007</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="27" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="28" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="52" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="53" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="54" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="55" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="56" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="57" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="58" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="59" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="60" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="61" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="62" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="63" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="64" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="68" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="69" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="70" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="71" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="75" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="76" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="77" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="78" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="79" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="80" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="82" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="83" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="84" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="85" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="86" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="87" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="88" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="89" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="90" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="91" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="92" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="93" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="94" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="95" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="96" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="97" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="98" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="99" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="100" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="101" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="102" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="103" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="104" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="105" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="106" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="107" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="108" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="109" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="110" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="111" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="112" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="113" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="114" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="115" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="116" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="117" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="118" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="119" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="120" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="121" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="122" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="123" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="124" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="125" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="126" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="127" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="128" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="129" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="130" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="131" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="132" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="133" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="134" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="135" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="136" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="137" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="138" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="139" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="140" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="141" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="142" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="143" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="144" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="145" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="146" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="147" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="148" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="149" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="150" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="151" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="152" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="153" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="154" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="155" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="156" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="157" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="158" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="159" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="160" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="161" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="162" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="163" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="164" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="165" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="166" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="167" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="168" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="169" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="170" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="171" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="172" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="173" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="174" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="175" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="176" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="177" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="178" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="179" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="180" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="181" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="182" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="183" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="184" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="185" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="186" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="187" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="188" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="189" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="190" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="191" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="192" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="193" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="194" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="195" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="196" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="197" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="198" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="199" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="200" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="201" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="202" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="203" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="204" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="205" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="206" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="207" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="208" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="209" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="210" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="211" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="212" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="213" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="214" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="215" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="216" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="220" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="221" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="222" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="223" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="224" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="225" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="226" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="227" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="228" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="229" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="230" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="231" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="232" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="233" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="234" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="235" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="236" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="237" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="238" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="239" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="240" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="241" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="242" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="243" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="244" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="245" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="246" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="247" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="248" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="249" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="250" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="251" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="252" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="253" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="254" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="255" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="256" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="257" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="258" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="259" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="260" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="261" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="262" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="263" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="264" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="265" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="266" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="267" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="268" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="269" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="270" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="271" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="272" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="273" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="274" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="275" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="276" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="277" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="278" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="279" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="280" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="281" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="282" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="283" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="284" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="285" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="286" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="287" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="288" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="289" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="290" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="291" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="292" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="293" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="294" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="295" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="296" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="297" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="298" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="299" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="300" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="301" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="302" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="303" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="304" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="305" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="306" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="307" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="308" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="309" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="310" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="311" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="312" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="313" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="314" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="315" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="316" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="317" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="318" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="319" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="320" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="321" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="322" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="323" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="324" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="325" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="326" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="327" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="328" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="329" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="330" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="331" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="332" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="333" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="334" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="335" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="336" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="337" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="338" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="339" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="340" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="341" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="342" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="343" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="344" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="345" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="346" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="347" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="348" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="349" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="350" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="351" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="352" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="353" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="354" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="355" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="356" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="357" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="358" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="359" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="360" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="361" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="362" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="363" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="364" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="365" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="366" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="367" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="368" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="369" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="370" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="371" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="372" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="373" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="374" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="375" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="376" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="377" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="378" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="379" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="380" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="381" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="382" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="383" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="384" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="385" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="386" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="387" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="388" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="389" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="390" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="391" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="392" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="393" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="394" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="395" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="396" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="397" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="398" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="399" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="400" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="401" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="402" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="403" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="404" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="405" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="406" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="407" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="408" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="409" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="410" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="411" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="412" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="413" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="414" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="415" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="416" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="417" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="418" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="419" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="420" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="421" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="422" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="423" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="424" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="425" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="426" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="427" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="428" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="429" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="430" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="431" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="432" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="433" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="434" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="435" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="436" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="437" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="438" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="439" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="440" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="441" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="442" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="443" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="444" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="445" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="446" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="447" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="448" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="449" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="450" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="451" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="452" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="453" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="454" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="455" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="456" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="457" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="458" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="459" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="460" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="461" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="462" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="463" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="464" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="465" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="466" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="467" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="468" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="469" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="470" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="471" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="472" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="473" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="474" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="475" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="476" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="477" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="478" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="479" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="480" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="481" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="482" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="483" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="484" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="485" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="486" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="487" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="488" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="489" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="490" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="491" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="492" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="493" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="494" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="495" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="496" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="497" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="498" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="499" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="500" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="501" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="502" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="503" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="504" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="505" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="506" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="507" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="508" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="509" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="510" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="511" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="512" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="513" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="514" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="515" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="516" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="517" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="518" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="519" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="520" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="521" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="522" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="523" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="524" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="525" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="526" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="527" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="528" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="529" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="530" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="531" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="532" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="533" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="534" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="535" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="536" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="537" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="538" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="539" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="540" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="541" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="542" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="543" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="544" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="545" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="546" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="547" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="548" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="549" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="550" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="551" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="552" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="553" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="554" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="555" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="556" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="557" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="558" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="559" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="560" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="561" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="562" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="563" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="564" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="565" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="566" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="567" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="568" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="569" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="570" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="571" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="572" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="573" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="574" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="575" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="576" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="577" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="578" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="579" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="580" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="581" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="582" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="583" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="584" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="585" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="586" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="587" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="588" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="589" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="590" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="591" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="592" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="593" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="594" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="595" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="596" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="597" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="598" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="599" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="600" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="601" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="602" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="603" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="604" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="605" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="606" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="607" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="608" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="609" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="610" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="611" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="612" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="613" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="614" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="615" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="616" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="617" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="618" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="619" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="620" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="621" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="622" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="623" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="624" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="625" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="626" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="627" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="628" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="629" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="630" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="631" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="632" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="633" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="634" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="635" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="636" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="637" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="638" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="639" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="640" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="641" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="642" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="643" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="644" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="645" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="646" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="647" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="648" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="649" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="650" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="651" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="652" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="653" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="654" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="655" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="656" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="657" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="658" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="659" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="660" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="661" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="662" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="663" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="664" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="665" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="666" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="667" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="668" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="669" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="670" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="671" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="672" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="673" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="674" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="675" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="676" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="677" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="678" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="679" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="680" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="681" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="682" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="683" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="684" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="685" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="686" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="687" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="688" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="689" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="690" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="691" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="692" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="693" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="694" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="695" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="696" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="697" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="698" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="699" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="700" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="701" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="702" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="703" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="704" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="705" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="706" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="707" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="708" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="709" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="710" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="711" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="712" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="713" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="714" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="715" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="716" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="717" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="718" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="719" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="720" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="721" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="722" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="723" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="724" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="725" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="726" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="727" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="728" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="729" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="730" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="731" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="732" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="733" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="734" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="735" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="736" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="737" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="738" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="739" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="740" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="741" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="742" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="743" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="744" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="745" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="746" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="747" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="748" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="749" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="750" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="751" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="752" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="753" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="754" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="755" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="756" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="757" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="758" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="759" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="760" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="761" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="762" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="763" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="764" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="765" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="766" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="767" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="768" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="769" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="770" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="771" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="772" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="773" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="774" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="775" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="776" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="777" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="778" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="779" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="780" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="781" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="782" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="783" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="784" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="785" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="786" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="787" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="788" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="789" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="790" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="791" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="792" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="793" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="794" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="795" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="796" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="797" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="798" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="799" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="800" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="801" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="802" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="803" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="804" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="805" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="806" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="807" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="808" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="809" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="810" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="811" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="812" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="813" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="814" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="815" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="816" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="817" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="818" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="819" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="820" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="821" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="822" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="823" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="824" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="825" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="826" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="827" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="828" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="829" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="830" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="831" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="832" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="833" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="834" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="835" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="836" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="837" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="838" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="839" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="840" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="841" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="842" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="843" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="844" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="845" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="846" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="847" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="848" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="849" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="850" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="851" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="852" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="853" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="854" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="855" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="856" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="857" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="858" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="859" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="860" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="861" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="862" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="863" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="864" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="865" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="866" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="867" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="868" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="869" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="870" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="871" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="872" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="873" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="874" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="875" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="876" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="877" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="878" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="879" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="880" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="881" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="882" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="883" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="884" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="885" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="886" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="887" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="888" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="889" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="890" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="891" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="892" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="893" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="894" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="895" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="896" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="897" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="898" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="899" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="900" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="901" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="902" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="903" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="904" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="905" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="906" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="907" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="908" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="909" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="910" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="911" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="912" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="913" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="914" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="915" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="916" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="917" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="918" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="919" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="920" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="921" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="922" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="923" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="924" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="925" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="926" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="927" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="928" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="929" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="930" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="931" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="932" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="933" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="934" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="935" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="936" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="937" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="938" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="939" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="940" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="941" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="942" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="943" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="944" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="945" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="946" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="947" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="948" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="949" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="950" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="951" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="952" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="953" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="954" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="955" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="956" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="957" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="958" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="959" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="960" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="961" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="962" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="963" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="964" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="965" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="966" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="967" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="968" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="969" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="970" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="971" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="972" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="973" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="974" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="975" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="976" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="977" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="978" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="979" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="980" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="981" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="982" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="983" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="984" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="985" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="986" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="987" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="988" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="989" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="990" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="991" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="992" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="993" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[SCRUM MASTER] Updated all the documents regarding Sprint 5. This concludes this sprint.
</commit_message>
<xml_diff>
--- a/SE202526/Management/Burndown Chart.xlsx
+++ b/SE202526/Management/Burndown Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilh\Documents\Universidade\ES\Projeto\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3900FA-4D84-4E49-8762-D8051B0A6729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EC29B2-6923-4823-A584-F61BF2DC7078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -124,13 +124,13 @@
     </r>
   </si>
   <si>
-    <t>Analyze the code relative to the two first User Stories</t>
+    <t>Produce videos/tests and documentation</t>
   </si>
   <si>
-    <t>Implement User Stories 1 and 2</t>
+    <t>Implement User Stories 1, 2 and 3</t>
   </si>
   <si>
-    <t>Produce videos/tests and documentation</t>
+    <t>Analyze the code relative to the User Stories</t>
   </si>
 </sst>
 </file>
@@ -692,27 +692,6 @@
   </cellStyleXfs>
   <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -847,6 +826,27 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1807,25 +1807,25 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1969,31 +1969,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0" formatCode="General">
-                  <c:v>19</c:v>
+                  <c:v>68</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16</c:v>
+                  <c:v>63</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>27.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3</c:v>
+                  <c:v>16.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3</c:v>
+                  <c:v>-1.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3</c:v>
+                  <c:v>-1.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2113,31 +2113,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0" formatCode="General">
-                  <c:v>19</c:v>
+                  <c:v>68</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.100000000000001</c:v>
+                  <c:v>61.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15.2</c:v>
+                  <c:v>54.4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13.3</c:v>
+                  <c:v>47.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11.4</c:v>
+                  <c:v>40.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9.5</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7.6000000000000014</c:v>
+                  <c:v>27.200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.7000000000000011</c:v>
+                  <c:v>20.399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.8000000000000007</c:v>
+                  <c:v>13.600000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2629,474 +2629,474 @@
   <sheetData>
     <row r="1" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
     </row>
     <row r="3" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="12"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="5"/>
     </row>
     <row r="4" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="7">
         <v>45961</v>
       </c>
-      <c r="F4" s="14">
+      <c r="F4" s="7">
         <v>45962</v>
       </c>
-      <c r="G4" s="14">
+      <c r="G4" s="7">
         <v>45963</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="7">
         <v>45964</v>
       </c>
-      <c r="I4" s="14">
+      <c r="I4" s="7">
         <v>45965</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="8">
         <v>45966</v>
       </c>
-      <c r="K4" s="14">
+      <c r="K4" s="7">
         <v>45967</v>
       </c>
-      <c r="L4" s="16">
+      <c r="L4" s="9">
         <v>45968</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="5"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="17" t="s">
+      <c r="B5" s="52"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="18" t="s">
+      <c r="I5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="18" t="s">
+      <c r="K5" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="13" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="21">
+      <c r="B6" s="14">
         <v>1</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="16">
         <v>1</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="17">
         <v>0.2</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="17">
         <v>0.2</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="17">
         <v>0.2</v>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="17">
         <v>0.4</v>
       </c>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="26"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="19"/>
     </row>
     <row r="7" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="27">
+      <c r="B7" s="20">
         <v>2</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="22">
         <v>3</v>
       </c>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30">
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23">
         <v>0.2</v>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="23">
         <v>0.4</v>
       </c>
-      <c r="I7" s="30">
+      <c r="I7" s="23">
         <v>0.6</v>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="24">
         <v>0.8</v>
       </c>
-      <c r="K7" s="30">
+      <c r="K7" s="23">
         <v>1</v>
       </c>
-      <c r="L7" s="32"/>
+      <c r="L7" s="25"/>
     </row>
     <row r="8" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="27">
+      <c r="B8" s="20">
         <v>3</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="22">
         <v>1</v>
       </c>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="31">
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="24">
         <v>1</v>
       </c>
-      <c r="K8" s="30"/>
-      <c r="L8" s="32"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="25"/>
     </row>
     <row r="9" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="27">
+      <c r="B9" s="20">
         <v>4</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="22">
         <v>2</v>
       </c>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="30">
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="23">
         <v>2</v>
       </c>
-      <c r="L9" s="32"/>
+      <c r="L9" s="25"/>
     </row>
     <row r="10" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="27">
+      <c r="B10" s="20">
         <v>5</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="22">
         <v>1</v>
       </c>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="32">
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="25">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="27">
+      <c r="B11" s="20">
         <v>6</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="32"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="25"/>
     </row>
     <row r="12" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="27">
+      <c r="B12" s="20">
         <v>7</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="32"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="25"/>
     </row>
     <row r="13" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="27">
+      <c r="B13" s="20">
         <v>8</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="30"/>
-      <c r="L13" s="32"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="25"/>
     </row>
     <row r="14" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="27">
+      <c r="B14" s="20">
         <v>9</v>
       </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="32"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="25"/>
     </row>
     <row r="15" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="27">
+      <c r="B15" s="20">
         <v>10</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="31"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="32"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="25"/>
     </row>
     <row r="16" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="27">
+      <c r="B16" s="20">
         <v>11</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="32"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="25"/>
     </row>
     <row r="17" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="27">
+      <c r="B17" s="20">
         <v>12</v>
       </c>
-      <c r="C17" s="34"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="30"/>
-      <c r="L17" s="32"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="25"/>
     </row>
     <row r="18" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="27">
+      <c r="B18" s="20">
         <v>13</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="32"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="25"/>
     </row>
     <row r="19" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="36">
+      <c r="B19" s="29">
         <v>14</v>
       </c>
-      <c r="C19" s="37"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
-      <c r="I19" s="39"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="39"/>
-      <c r="L19" s="41"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="42">
+      <c r="C20" s="54"/>
+      <c r="D20" s="35">
         <v>0</v>
       </c>
-      <c r="E20" s="43">
+      <c r="E20" s="36">
         <f t="shared" ref="E20:L20" si="0">SUM(E6:E19)</f>
         <v>0.2</v>
       </c>
-      <c r="F20" s="43">
+      <c r="F20" s="36">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="36">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="H20" s="43">
+      <c r="H20" s="36">
         <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
-      <c r="I20" s="43">
+      <c r="I20" s="36">
         <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
-      <c r="J20" s="44">
+      <c r="J20" s="37">
         <f t="shared" si="0"/>
         <v>1.8</v>
       </c>
-      <c r="K20" s="44">
+      <c r="K20" s="37">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="L20" s="45">
+      <c r="L20" s="38">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="46">
+      <c r="C21" s="48"/>
+      <c r="D21" s="39">
         <f>SUM(D6:D20)</f>
         <v>8</v>
       </c>
-      <c r="E21" s="47">
+      <c r="E21" s="40">
         <f t="shared" ref="E21:L21" si="1">D21-SUM(E6:E19)</f>
         <v>7.8</v>
       </c>
-      <c r="F21" s="47">
+      <c r="F21" s="40">
         <f t="shared" si="1"/>
         <v>7.6</v>
       </c>
-      <c r="G21" s="47">
+      <c r="G21" s="40">
         <f t="shared" si="1"/>
         <v>7.1999999999999993</v>
       </c>
-      <c r="H21" s="47">
+      <c r="H21" s="40">
         <f t="shared" si="1"/>
         <v>6.3999999999999995</v>
       </c>
-      <c r="I21" s="47">
+      <c r="I21" s="40">
         <f t="shared" si="1"/>
         <v>5.8</v>
       </c>
-      <c r="J21" s="48">
+      <c r="J21" s="41">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="K21" s="49">
+      <c r="K21" s="42">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="L21" s="50">
+      <c r="L21" s="43">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="51">
+      <c r="C22" s="49"/>
+      <c r="D22" s="44">
         <f>D21</f>
         <v>8</v>
       </c>
-      <c r="E22" s="52">
+      <c r="E22" s="45">
         <f>$D$22-($D$22/10*1)</f>
         <v>7.2</v>
       </c>
-      <c r="F22" s="52">
+      <c r="F22" s="45">
         <f>$D$22-($D$22/10*2)</f>
         <v>6.4</v>
       </c>
-      <c r="G22" s="52">
+      <c r="G22" s="45">
         <f>$D$22-($D$22/10*3)</f>
         <v>5.6</v>
       </c>
-      <c r="H22" s="52">
+      <c r="H22" s="45">
         <f>$D$22-($D$22/10*4)</f>
         <v>4.8</v>
       </c>
-      <c r="I22" s="52">
+      <c r="I22" s="45">
         <f>$D$22-($D$22/10*5)</f>
         <v>4</v>
       </c>
-      <c r="J22" s="53">
+      <c r="J22" s="46">
         <f>$D$22-($D$22/10*6)</f>
         <v>3.1999999999999993</v>
       </c>
-      <c r="K22" s="52">
+      <c r="K22" s="45">
         <f>$D$22-($D$22/10*7)</f>
         <v>2.3999999999999995</v>
       </c>
-      <c r="L22" s="54">
+      <c r="L22" s="47">
         <f>$D$22-($D$22/10*8)</f>
         <v>1.5999999999999996</v>
       </c>
@@ -4097,472 +4097,488 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDEF1E91-1F52-494C-B1A2-6E397623B912}">
-  <dimension ref="B1:L1000"/>
+  <dimension ref="B1:M1000"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" customWidth="1"/>
     <col min="2" max="2" width="7.1796875" customWidth="1"/>
     <col min="3" max="3" width="73.08984375" customWidth="1"/>
     <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="14" width="10" customWidth="1"/>
+    <col min="5" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="10" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
     <col min="15" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
     </row>
     <row r="3" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="12"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="5"/>
     </row>
     <row r="4" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="7">
         <v>45979</v>
       </c>
-      <c r="F4" s="14">
+      <c r="F4" s="7">
         <v>45980</v>
       </c>
-      <c r="G4" s="14">
+      <c r="G4" s="7">
         <v>45981</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="7">
         <v>45982</v>
       </c>
-      <c r="I4" s="14">
+      <c r="I4" s="7">
         <v>45983</v>
       </c>
-      <c r="J4" s="14">
+      <c r="J4" s="7">
         <v>45984</v>
       </c>
-      <c r="K4" s="14">
+      <c r="K4" s="7">
         <v>45985</v>
       </c>
-      <c r="L4" s="14">
+      <c r="L4" s="7">
         <v>45986</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="5"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="17" t="s">
+      <c r="B5" s="52"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="18" t="s">
+      <c r="I5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="18" t="s">
+      <c r="K5" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="13" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="21">
+      <c r="B6" s="14">
         <v>1</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="23">
-        <v>6</v>
-      </c>
-      <c r="E6" s="24">
-        <v>1</v>
-      </c>
-      <c r="F6" s="24">
+      <c r="C6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="16">
+        <v>10</v>
+      </c>
+      <c r="E6" s="17">
         <v>3</v>
       </c>
-      <c r="G6" s="24">
-        <v>2</v>
-      </c>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="26"/>
+      <c r="F6" s="17">
+        <v>3</v>
+      </c>
+      <c r="G6" s="17">
+        <v>4</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="19"/>
     </row>
     <row r="7" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="27">
+      <c r="B7" s="20">
         <v>2</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="29">
-        <v>7</v>
-      </c>
-      <c r="E7" s="30">
+      <c r="D7" s="22">
+        <v>48</v>
+      </c>
+      <c r="E7" s="23">
         <v>2</v>
       </c>
-      <c r="F7" s="30">
-        <v>3</v>
-      </c>
-      <c r="G7" s="30">
+      <c r="F7" s="23">
         <v>5</v>
       </c>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="32"/>
+      <c r="G7" s="23">
+        <v>10</v>
+      </c>
+      <c r="H7" s="23">
+        <v>13</v>
+      </c>
+      <c r="I7" s="23">
+        <v>10</v>
+      </c>
+      <c r="J7" s="24">
+        <v>5</v>
+      </c>
+      <c r="K7" s="23">
+        <v>10</v>
+      </c>
+      <c r="L7" s="25"/>
     </row>
     <row r="8" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="27">
+      <c r="B8" s="20">
         <v>3</v>
       </c>
-      <c r="C8" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="29">
-        <v>4</v>
-      </c>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="32"/>
+      <c r="C8" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="22">
+        <v>6</v>
+      </c>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="I8" s="23">
+        <v>1</v>
+      </c>
+      <c r="J8" s="24">
+        <v>3</v>
+      </c>
+      <c r="K8" s="23"/>
+      <c r="L8" s="25"/>
     </row>
     <row r="9" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="27">
+      <c r="B9" s="20">
         <v>4</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="29">
-        <v>2</v>
-      </c>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="32"/>
+      <c r="D9" s="22">
+        <v>4</v>
+      </c>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="25"/>
     </row>
     <row r="10" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="27">
+      <c r="B10" s="20">
         <v>5</v>
       </c>
-      <c r="D10" s="29"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="32"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="25"/>
     </row>
     <row r="11" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="27">
+      <c r="B11" s="20">
         <v>6</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="32"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="25"/>
     </row>
     <row r="12" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="27">
+      <c r="B12" s="20">
         <v>7</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="32"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="25"/>
     </row>
     <row r="13" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="27">
+      <c r="B13" s="20">
         <v>8</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="30"/>
-      <c r="L13" s="32"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="25"/>
     </row>
     <row r="14" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="27">
+      <c r="B14" s="20">
         <v>9</v>
       </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="32"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="25"/>
     </row>
     <row r="15" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="27">
+      <c r="B15" s="20">
         <v>10</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="31"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="32"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="25"/>
     </row>
     <row r="16" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="27">
+      <c r="B16" s="20">
         <v>11</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="32"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="25"/>
     </row>
     <row r="17" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="27">
+      <c r="B17" s="20">
         <v>12</v>
       </c>
-      <c r="C17" s="34"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="30"/>
-      <c r="L17" s="32"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="25"/>
     </row>
     <row r="18" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="27">
+      <c r="B18" s="20">
         <v>13</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="32"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="25"/>
     </row>
     <row r="19" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="36">
+      <c r="B19" s="29">
         <v>14</v>
       </c>
-      <c r="C19" s="37"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
-      <c r="I19" s="39"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="39"/>
-      <c r="L19" s="41"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="42">
+      <c r="C20" s="54"/>
+      <c r="D20" s="35">
         <v>0</v>
       </c>
-      <c r="E20" s="43">
+      <c r="E20" s="36">
         <f t="shared" ref="E20:L20" si="0">SUM(E6:E19)</f>
-        <v>3</v>
-      </c>
-      <c r="F20" s="43">
+        <v>5</v>
+      </c>
+      <c r="F20" s="36">
         <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="G20" s="43">
+        <v>8</v>
+      </c>
+      <c r="G20" s="36">
         <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="H20" s="43">
+        <v>14</v>
+      </c>
+      <c r="H20" s="36">
+        <f t="shared" si="0"/>
+        <v>13.5</v>
+      </c>
+      <c r="I20" s="36">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="J20" s="37">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="K20" s="37">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="L20" s="38">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I20" s="43">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J20" s="44">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K20" s="44">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L20" s="45">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
     </row>
     <row r="21" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="46">
+      <c r="C21" s="48"/>
+      <c r="D21" s="39">
         <f>SUM(D6:D20)</f>
-        <v>19</v>
-      </c>
-      <c r="E21" s="47">
+        <v>68</v>
+      </c>
+      <c r="E21" s="40">
         <f t="shared" ref="E21:L21" si="1">D21-SUM(E6:E19)</f>
-        <v>16</v>
-      </c>
-      <c r="F21" s="47">
+        <v>63</v>
+      </c>
+      <c r="F21" s="40">
         <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="G21" s="47">
+        <v>55</v>
+      </c>
+      <c r="G21" s="40">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="H21" s="47">
+        <v>41</v>
+      </c>
+      <c r="H21" s="40">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="I21" s="47">
+        <v>27.5</v>
+      </c>
+      <c r="I21" s="40">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="J21" s="48">
+        <v>16.5</v>
+      </c>
+      <c r="J21" s="41">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="K21" s="49">
+        <v>8.5</v>
+      </c>
+      <c r="K21" s="42">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="L21" s="50">
+        <v>-1.5</v>
+      </c>
+      <c r="L21" s="43">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="22" spans="2:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="51">
+      <c r="C22" s="49"/>
+      <c r="D22" s="44">
         <f>D21</f>
-        <v>19</v>
-      </c>
-      <c r="E22" s="52">
+        <v>68</v>
+      </c>
+      <c r="E22" s="45">
         <f>$D$22-($D$22/10*1)</f>
-        <v>17.100000000000001</v>
-      </c>
-      <c r="F22" s="52">
+        <v>61.2</v>
+      </c>
+      <c r="F22" s="45">
         <f>$D$22-($D$22/10*2)</f>
-        <v>15.2</v>
-      </c>
-      <c r="G22" s="52">
+        <v>54.4</v>
+      </c>
+      <c r="G22" s="45">
         <f>$D$22-($D$22/10*3)</f>
-        <v>13.3</v>
-      </c>
-      <c r="H22" s="52">
+        <v>47.6</v>
+      </c>
+      <c r="H22" s="45">
         <f>$D$22-($D$22/10*4)</f>
-        <v>11.4</v>
-      </c>
-      <c r="I22" s="52">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="I22" s="45">
         <f>$D$22-($D$22/10*5)</f>
-        <v>9.5</v>
-      </c>
-      <c r="J22" s="53">
+        <v>34</v>
+      </c>
+      <c r="J22" s="46">
         <f>$D$22-($D$22/10*6)</f>
-        <v>7.6000000000000014</v>
-      </c>
-      <c r="K22" s="52">
+        <v>27.200000000000003</v>
+      </c>
+      <c r="K22" s="45">
         <f>$D$22-($D$22/10*7)</f>
-        <v>5.7000000000000011</v>
-      </c>
-      <c r="L22" s="54">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="L22" s="47">
         <f>$D$22-($D$22/10*8)</f>
-        <v>3.8000000000000007</v>
+        <v>13.600000000000001</v>
       </c>
     </row>
     <row r="23" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>

</xml_diff>